<commit_message>
.gitignore is now working
</commit_message>
<xml_diff>
--- a/XD_JIG/XD04/XD04_PWM_Rev_0/Docs/LTC6102_Param.xlsx
+++ b/XD_JIG/XD04/XD04_PWM_Rev_0/Docs/LTC6102_Param.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\Jig\XD_JIG\XD04\XD04_PWM_Rev_0\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A53281A-DA6B-456E-A8D3-5775D49E7CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{785817AA-981A-4C2E-A1CC-0DA5CFBAF76E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4620" yWindow="293" windowWidth="16050" windowHeight="12764" activeTab="1" xr2:uid="{11FFDA7F-9C68-49B0-9D76-D5DA7C94FBB9}"/>
+    <workbookView xWindow="43080" yWindow="4095" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{11FFDA7F-9C68-49B0-9D76-D5DA7C94FBB9}"/>
   </bookViews>
   <sheets>
     <sheet name="Org" sheetId="1" r:id="rId1"/>
@@ -341,7 +341,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="18">
+  <numFmts count="19">
     <numFmt numFmtId="176" formatCode="0&quot;mA&quot;"/>
     <numFmt numFmtId="177" formatCode="0.000&quot;V&quot;"/>
     <numFmt numFmtId="178" formatCode="0.0&quot;mA&quot;"/>
@@ -360,6 +360,7 @@
     <numFmt numFmtId="191" formatCode="0.00000&quot;V&quot;"/>
     <numFmt numFmtId="192" formatCode="0.0000000&quot;V&quot;"/>
     <numFmt numFmtId="193" formatCode="0.0&quot;Ω&quot;"/>
+    <numFmt numFmtId="209" formatCode="0.000000000_);[Red]\(0.000000000\)"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -417,7 +418,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -500,6 +501,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="209" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3171,7 +3175,7 @@
   <cols>
     <col min="1" max="1" width="2.625" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.3125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.75" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.25" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.125" style="1" bestFit="1" customWidth="1"/>
@@ -5075,6 +5079,10 @@
       </c>
     </row>
     <row r="28" spans="2:27" x14ac:dyDescent="0.6">
+      <c r="C28" s="28">
+        <f>E9/D3</f>
+        <v>2.5247130566506768E-5</v>
+      </c>
       <c r="P28" s="17"/>
       <c r="Q28" s="17"/>
       <c r="R28" s="17"/>

</xml_diff>